<commit_message>
Prepared demo data with one sample member
</commit_message>
<xml_diff>
--- a/backend/global_members.xlsx
+++ b/backend/global_members.xlsx
@@ -118,10 +118,10 @@
     <t>West Nyack</t>
   </si>
   <si>
-    <t>ajay.avasatthi</t>
-  </si>
-  <si>
     <t xml:space="preserve"> LEN-GG45AA</t>
+  </si>
+  <si>
+    <t>ajay11</t>
   </si>
 </sst>
 </file>
@@ -606,16 +606,16 @@
         <v>22</v>
       </c>
       <c r="S2" t="s">
+        <v>34</v>
+      </c>
+      <c r="T2" t="s">
         <v>35</v>
-      </c>
-      <c r="T2" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:U1 A2:Q2 T2:U2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:U1 A2:Q2 U2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>